<commit_message>
Update the consistency check tables
</commit_message>
<xml_diff>
--- a/Data/Results/From Clean Raw Data/Step 3_2026 Format/SIC Codes Consistency Check_Buddhist_08.15.2026.xlsx
+++ b/Data/Results/From Clean Raw Data/Step 3_2026 Format/SIC Codes Consistency Check_Buddhist_08.15.2026.xlsx
@@ -17,29 +17,44 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="25">
   <si>
     <t>x</t>
   </si>
   <si>
+    <t>classifier</t>
+  </si>
+  <si>
     <t>Freq</t>
   </si>
   <si>
     <t>TEMPLES-BUDDHIST</t>
   </si>
   <si>
+    <t>Buddhist Temple</t>
+  </si>
+  <si>
     <t>CHURCHES</t>
   </si>
   <si>
+    <t>Christian Church; Interfaith</t>
+  </si>
+  <si>
     <t>SYNAGOGUES</t>
   </si>
   <si>
+    <t>Jewish Synagogue</t>
+  </si>
+  <si>
     <t>CHURCH ORGANIZATIONS</t>
   </si>
   <si>
     <t>CONVENTS &amp; MONASTERIES</t>
   </si>
   <si>
+    <t>Interfaith</t>
+  </si>
+  <si>
     <t>MEDITATION ORGANIZATIONS</t>
   </si>
   <si>
@@ -49,6 +64,9 @@
     <t>TEMPLES-HINDU</t>
   </si>
   <si>
+    <t>Hindu Mandir</t>
+  </si>
+  <si>
     <t>CLERGY</t>
   </si>
   <si>
@@ -68,6 +86,9 @@
   </si>
   <si>
     <t>SPIRITUAL ORGANIZATIONS</t>
+  </si>
+  <si>
+    <t>Other Religion</t>
   </si>
   <si>
     <t>SYNAGOGUES JEWISH</t>
@@ -413,22 +434,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
     </row>
@@ -439,78 +466,105 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
         <v>0.462</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
         <v>0.406</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
         <v>0.08500000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5">
         <v>0.008999999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6">
         <v>0.008999999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
         <v>0.008999999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8">
         <v>0.008999999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
         <v>0.008999999999999999</v>
       </c>
     </row>
@@ -521,62 +575,83 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2">
+        <v>0.392</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>0.381</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
-        <v>0.392</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>0.381</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+      <c r="C4">
         <v>0.175</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
         <v>0.021</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6">
         <v>0.021</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
         <v>0.01</v>
       </c>
     </row>
@@ -587,142 +662,193 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1">
+    <row r="1" spans="1:3" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
         <v>0.385</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
         <v>0.377</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4">
         <v>0.155</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>0.057</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7">
+        <v>0.005</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>0.004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9">
+        <v>0.003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>0.002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15">
+        <v>0.001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
         <v>8</v>
       </c>
-      <c r="B5">
-        <v>0.057</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>0.005</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8">
-        <v>0.004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9">
-        <v>0.003</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10">
-        <v>0.002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11">
+      <c r="C16">
         <v>0.001</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
         <v>14</v>
       </c>
-      <c r="B13">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+      <c r="B17" t="s">
         <v>15</v>
       </c>
-      <c r="B14">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16">
-        <v>0.001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17">
+      <c r="C17">
         <v>0.001</v>
       </c>
     </row>

</xml_diff>